<commit_message>
Split invocation from genealogy preamble into dedicated column
Add _extract_invocation() which splits on 'and may' to isolate the
invocation clause from the author genealogy ('By X son of Y...').

Column order is now: Category | Invocation (English) | Full Translation |
Safaitic Text (Transliteration) — giving a clean two-column invocation+
category view while preserving the complete text alongside.

https://claude.ai/code/session_01HBAq6ujN3GER4UH7qmYUUk
</commit_message>
<xml_diff>
--- a/safaitic-research/safaitic_invocations.xlsx
+++ b/safaitic-research/safaitic_invocations.xlsx
@@ -660,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -669,7 +669,8 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -695,15 +696,20 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Invocation (English)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Full Translation</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Safaitic Text (Transliteration)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>English Translation</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Source File</t>
         </is>
@@ -732,15 +738,20 @@
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
+          <t>And may Allāt take vengeance on whoever did evil against him.</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>By Nṣr son of Ṣlt son of ʿMr, and may Allāt take vengeance on whoever did evil against him.</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
           <t>l-nṣr bn ṣlt bn ʿmr w-h-Allāt nqm mn fʿl bh s²r</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
-        <is>
-          <t>By Nṣr son of Ṣlt son of ʿMr, and may Allāt take vengeance on whoever did evil against him.</t>
-        </is>
-      </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>USMF0002.xml</t>
         </is>
@@ -769,15 +780,20 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
+          <t>And may Allāt (grant) protection and peace and help.</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>By Khl son of Šʿd son of Ḥwš, and may Allāt (grant) protection and peace and help.</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
           <t>l-khl bn s²ʿd bn ḥwš w-h-Allāt ḥmyt w-slm w-ʿwn</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>By Khl son of Šʿd son of Ḥwš, and may Allāt (grant) protection and peace and help.</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>RSIS0003.xml</t>
         </is>
@@ -806,15 +822,20 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
+          <t>And may Rudā take vengeance on every enemy.</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>By Slm son of ʿMt son of Hfʿl, and may Rudā take vengeance on every enemy.</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
           <t>l-Slm bn ʿmt bn hfʿl w-nqm h-Rudā mn kl ʿdw</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>By Slm son of ʿMt son of Hfʿl, and may Rudā take vengeance on every enemy.</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>KRS0002.xml</t>
         </is>
@@ -843,15 +864,20 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
+          <t>And may Allāt (grant) protection, and may Rudā take vengeance on his enemy, and may Shams (grant) rain and good pasture.</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>By Ṣhr son of Sʿd son of Ṯlm, and may Allāt (grant) protection, and may Rudā take vengeance on his enemy, and may Shams (grant) rain and good pasture.</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
           <t>l-ṣhr bn s¹ʿd bn ṯlm w-h-Allāt ḥmyt w-h-Rudā nqm mn s²nʾ-h w-h-Šms gyt w-mrʿ</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>By Ṣhr son of Sʿd son of Ṯlm, and may Allāt (grant) protection, and may Rudā take vengeance on his enemy, and may Shams (grant) rain and good pasture.</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>USMF0003.xml</t>
         </is>
@@ -880,15 +906,20 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
+          <t>And may Allāt (grant) protection, and may Rudā take vengeance for him on his enemy, and may Shams (grant) good pasture.</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>By Ḥry son of ʿMr son of ʿBd, and may Allāt (grant) protection, and may Rudā take vengeance for him on his enemy, and may Shams (grant) good pasture.</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
           <t>l-ḥry bn ʿmr bn ʿbd w-h-Allāt ḥmyt w-h-Rudā nqm l-h mn ʿdw-h w-h-Šms mrʿ</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>By Ḥry son of ʿMr son of ʿBd, and may Allāt (grant) protection, and may Rudā take vengeance for him on his enemy, and may Shams (grant) good pasture.</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>KRS0003.xml</t>
         </is>
@@ -917,15 +948,20 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
+          <t>And may Shams grant him good fortune and (good) pasture and rain.</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>By ʿWr son of Ngr, and may Shams grant him good fortune and (good) pasture and rain.</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
           <t>l-ʿwr bn ngr w-h-Šms tns¹ʿd-h w-mrʿ w-wbl</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>By ʿWr son of Ngr, and may Shams grant him good fortune and (good) pasture and rain.</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>USMF0001.xml</t>
         </is>
@@ -954,15 +990,20 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
+          <t>And may Allāt protect him.</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>By Rḍw son of Ḥzm son of Ḥyw son of Ġwt, and may Allāt protect him.</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
           <t>b-s¹nt rḍw bn ḥzm bn ḥyw bn ġwt w-h-Allāt ḥmy-h</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>By Rḍw son of Ḥzm son of Ḥyw son of Ġwt, and may Allāt protect him.</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="H8" s="8" t="inlineStr">
         <is>
           <t>KRS0001.xml</t>
         </is>
@@ -991,15 +1032,20 @@
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
+          <t>And may Shams (grant) rain and good pasture for his camels.</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>By Sʿd son of Ġwt, while he pastured the camels, and may Shams (grant) rain and good pasture for his camels.</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
           <t>l-s¹ʿd bn ġwt w-rʿy h-ibl w-h-Šms gyt w-mrʿ l-ibl-h</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>By Sʿd son of Ġwt, while he pastured the camels, and may Shams (grant) rain and good pasture for his camels.</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="H9" s="9" t="inlineStr">
         <is>
           <t>HCH0002.xml</t>
         </is>
@@ -1028,15 +1074,20 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
+          <t>And may Shams (grant) good pasture and rain and gain, and may Allāt (grant) protection.</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>By ʿBd-Šms son of Mlk, while he pastured (flocks), and may Shams (grant) good pasture and rain and gain, and may Allāt (grant) protection.</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
           <t>l-ʿbd- Šms bn mlk w-rʿy w-h-Šms mrʿ w-wbl w-ks²b w-h-Allāt ḥmyt</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>By ʿBd-Šms son of Mlk, while he pastured (flocks), and may Shams (grant) good pasture and rain and gain, and may Allāt (grant) protection.</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>JDWS0002.xml</t>
         </is>
@@ -1065,15 +1116,20 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
+          <t>And may Rudā curse whoever erases this inscription.</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>By ʿBd son of Ḥnn, and may Rudā curse whoever erases this inscription.</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
           <t>l-ʿbd bn ḥnn w-h-Rudā lʿn mn mḥy h-ktbt</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>By ʿBd son of Ḥnn, and may Rudā curse whoever erases this inscription.</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="H11" s="9" t="inlineStr">
         <is>
           <t>WH0004.xml</t>
         </is>
@@ -1102,15 +1158,20 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
+          <t>And may Shams (grant) good pasture and rain.</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>By Ṯʿlbt son of Slm, while he pastured the sheep, and may Shams (grant) good pasture and rain.</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
           <t>l-ṯʿlbt bn s¹lm w-rʿy h-ġnm w-h-Šms mrʿ w-gyt</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>By Ṯʿlbt son of Slm, while he pastured the sheep, and may Shams (grant) good pasture and rain.</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr">
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>HCH0003.xml</t>
         </is>
@@ -1139,15 +1200,20 @@
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
+          <t>And may Rudā take retribution for him against his enemy.</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>By ʿMr son of Ḥnn, and may Rudā take retribution for him against his enemy.</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
           <t>l-ʿmr bn ḥnn w-h-Rudā ṯʾr-h mn ʿdw-h</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>By ʿMr son of Ḥnn, and may Rudā take retribution for him against his enemy.</t>
-        </is>
-      </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="H13" s="9" t="inlineStr">
         <is>
           <t>KRS0004.xml</t>
         </is>
@@ -1176,15 +1242,20 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
+          <t>And may Shams (grant) good pasture and rain and gain.</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>By Ġnm son of ʿMr, while he pastured (flocks), and may Shams (grant) good pasture and rain and gain.</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
           <t>l-ġnm bn ʿmr w-rʿy w-h-Šms mrʿ w-gyt w-ks²b</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>By Ġnm son of ʿMr, while he pastured (flocks), and may Shams (grant) good pasture and rain and gain.</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>WH0002.xml</t>
         </is>
@@ -1213,15 +1284,20 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
+          <t>And may Rudā take vengeance on his enemy.</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>By ʿMrt son of ʿBd son of Ḥrm, and may Rudā take vengeance on his enemy.</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
           <t>l-ʿmrt bn ʿbd bn ḥrm w-h-Rudā nqm mn s²nʾ-h</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>By ʿMrt son of ʿBd son of Ḥrm, and may Rudā take vengeance on his enemy.</t>
-        </is>
-      </c>
-      <c r="G15" s="9" t="inlineStr">
+      <c r="H15" s="9" t="inlineStr">
         <is>
           <t>RSIS0002.xml</t>
         </is>
@@ -1250,15 +1326,20 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
+          <t>And may Allāt protect him from every enemy, and may Shams (grant) pasture and gain.</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>By Ḥnn son of Ṣhr, and may Allāt protect him from every enemy, and may Shams (grant) pasture and gain.</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
           <t>l-ḥnn bn ṣhr w-h-Allāt ḥmy-h mn kl ʿdw w-h-Šms mrʿ w-ks²b</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>By Ḥnn son of Ṣhr, and may Allāt protect him from every enemy, and may Shams (grant) pasture and gain.</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
+      <c r="H16" s="8" t="inlineStr">
         <is>
           <t>RSIS0001.xml</t>
         </is>
@@ -1287,15 +1368,20 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
+          <t>And may Allāt take vengeance for him on his enemy, and may Rudā protect him.</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>By Ṯlm son of Ḫlf son of Šbq, and may Allāt take vengeance for him on his enemy, and may Rudā protect him.</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
           <t>l-ṯlm bn ḫlf bn s²bq w-h-Allāt nqm-h mn s²nʾ-h w-h-Rudā ḥmy-h</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>By Ṯlm son of Ḫlf son of Šbq, and may Allāt take vengeance for him on his enemy, and may Rudā protect him.</t>
-        </is>
-      </c>
-      <c r="G17" s="9" t="inlineStr">
+      <c r="H17" s="9" t="inlineStr">
         <is>
           <t>WH0003.xml</t>
         </is>
@@ -1324,15 +1410,20 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
+          <t>And may Shams save him and (grant) peace and help.</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>By Šrḥ son of ʿBd, and may Shams save him and (grant) peace and help.</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
           <t>l-s²rḥ bn ʿbd w-h-Šms ns²r-h w-slm w-ʿwn</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>By Šrḥ son of ʿBd, and may Shams save him and (grant) peace and help.</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
+      <c r="H18" s="8" t="inlineStr">
         <is>
           <t>JDWS0001.xml</t>
         </is>
@@ -1361,15 +1452,20 @@
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
+          <t>And may Allāt (grant) peace and protection.</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>By ʿbd-Allāt son of Šʿd son of Ġnm, and may Allāt (grant) peace and protection.</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
           <t>l-ʿbd- Allāt bn s²ʿd bn ġnm w-h-Allāt slm w-ḥmyt</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
-        <is>
-          <t>By ʿbd-Allāt son of Šʿd son of Ġnm, and may Allāt (grant) peace and protection.</t>
-        </is>
-      </c>
-      <c r="G19" s="9" t="inlineStr">
+      <c r="H19" s="9" t="inlineStr">
         <is>
           <t>WH0001.xml</t>
         </is>
@@ -1398,15 +1494,20 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
+          <t>And may Rudā protect him and help him.</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>By Wdm son of ʿWn son of Sʿd, and may Rudā protect him and help him.</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
           <t>l-wdm bn ʿwn bn s¹ʿd w-h-Rudā ḥmy-h w-ʿwn-h</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>By Wdm son of ʿWn son of Sʿd, and may Rudā protect him and help him.</t>
-        </is>
-      </c>
-      <c r="G20" s="8" t="inlineStr">
+      <c r="H20" s="8" t="inlineStr">
         <is>
           <t>HCH0001.xml</t>
         </is>
@@ -1423,7 +1524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1432,7 +1533,8 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1458,15 +1560,20 @@
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
+          <t>Invocation (English)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Full Translation</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
           <t>Safaitic Text (Transliteration)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>English Translation</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Source File</t>
         </is>
@@ -1495,15 +1602,20 @@
       </c>
       <c r="E2" s="10" t="inlineStr">
         <is>
+          <t>And may Allāt (grant) protection and peace and help.</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>By Khl son of Šʿd son of Ḥwš, and may Allāt (grant) protection and peace and help.</t>
+        </is>
+      </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
           <t>l-khl bn s²ʿd bn ḥwš w-h-Allāt ḥmyt w-slm w-ʿwn</t>
         </is>
       </c>
-      <c r="F2" s="10" t="inlineStr">
-        <is>
-          <t>By Khl son of Šʿd son of Ḥwš, and may Allāt (grant) protection and peace and help.</t>
-        </is>
-      </c>
-      <c r="G2" s="10" t="inlineStr">
+      <c r="H2" s="10" t="inlineStr">
         <is>
           <t>RSIS0003.xml</t>
         </is>
@@ -1532,15 +1644,20 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
+          <t>And may Allāt protect him.</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>By Rḍw son of Ḥzm son of Ḥyw son of Ġwt, and may Allāt protect him.</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
           <t>b-s¹nt rḍw bn ḥzm bn ḥyw bn ġwt w-h-Allāt ḥmy-h</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>By Rḍw son of Ḥzm son of Ḥyw son of Ġwt, and may Allāt protect him.</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>KRS0001.xml</t>
         </is>
@@ -1569,15 +1686,20 @@
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
+          <t>And may Shams save him and (grant) peace and help.</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>By Šrḥ son of ʿBd, and may Shams save him and (grant) peace and help.</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
           <t>l-s²rḥ bn ʿbd w-h-Šms ns²r-h w-slm w-ʿwn</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
-        <is>
-          <t>By Šrḥ son of ʿBd, and may Shams save him and (grant) peace and help.</t>
-        </is>
-      </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="H4" s="10" t="inlineStr">
         <is>
           <t>JDWS0001.xml</t>
         </is>
@@ -1606,15 +1728,20 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
+          <t>And may Allāt (grant) peace and protection.</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>By ʿbd-Allāt son of Šʿd son of Ġnm, and may Allāt (grant) peace and protection.</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
           <t>l-ʿbd- Allāt bn s²ʿd bn ġnm w-h-Allāt slm w-ḥmyt</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>By ʿbd-Allāt son of Šʿd son of Ġnm, and may Allāt (grant) peace and protection.</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>WH0001.xml</t>
         </is>
@@ -1643,15 +1770,20 @@
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
+          <t>And may Rudā protect him and help him.</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>By Wdm son of ʿWn son of Sʿd, and may Rudā protect him and help him.</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
           <t>l-wdm bn ʿwn bn s¹ʿd w-h-Rudā ḥmy-h w-ʿwn-h</t>
         </is>
       </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>By Wdm son of ʿWn son of Sʿd, and may Rudā protect him and help him.</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="H6" s="10" t="inlineStr">
         <is>
           <t>HCH0001.xml</t>
         </is>
@@ -1668,7 +1800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1677,7 +1809,8 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1703,15 +1836,20 @@
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
+          <t>Invocation (English)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Full Translation</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
           <t>Safaitic Text (Transliteration)</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>English Translation</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Source File</t>
         </is>
@@ -1740,15 +1878,20 @@
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
+          <t>And may Allāt take vengeance on whoever did evil against him.</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>By Nṣr son of Ṣlt son of ʿMr, and may Allāt take vengeance on whoever did evil against him.</t>
+        </is>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
           <t>l-nṣr bn ṣlt bn ʿmr w-h-Allāt nqm mn fʿl bh s²r</t>
         </is>
       </c>
-      <c r="F2" s="11" t="inlineStr">
-        <is>
-          <t>By Nṣr son of Ṣlt son of ʿMr, and may Allāt take vengeance on whoever did evil against him.</t>
-        </is>
-      </c>
-      <c r="G2" s="11" t="inlineStr">
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>USMF0002.xml</t>
         </is>
@@ -1777,15 +1920,20 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
+          <t>And may Rudā take vengeance on every enemy.</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>By Slm son of ʿMt son of Hfʿl, and may Rudā take vengeance on every enemy.</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
           <t>l-Slm bn ʿmt bn hfʿl w-nqm h-Rudā mn kl ʿdw</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>By Slm son of ʿMt son of Hfʿl, and may Rudā take vengeance on every enemy.</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>KRS0002.xml</t>
         </is>
@@ -1814,15 +1962,20 @@
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
+          <t>And may Rudā curse whoever erases this inscription.</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>By ʿBd son of Ḥnn, and may Rudā curse whoever erases this inscription.</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
           <t>l-ʿbd bn ḥnn w-h-Rudā lʿn mn mḥy h-ktbt</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
-        <is>
-          <t>By ʿBd son of Ḥnn, and may Rudā curse whoever erases this inscription.</t>
-        </is>
-      </c>
-      <c r="G4" s="11" t="inlineStr">
+      <c r="H4" s="11" t="inlineStr">
         <is>
           <t>WH0004.xml</t>
         </is>
@@ -1851,15 +2004,20 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
+          <t>And may Rudā take retribution for him against his enemy.</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>By ʿMr son of Ḥnn, and may Rudā take retribution for him against his enemy.</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
           <t>l-ʿmr bn ḥnn w-h-Rudā ṯʾr-h mn ʿdw-h</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>By ʿMr son of Ḥnn, and may Rudā take retribution for him against his enemy.</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>KRS0004.xml</t>
         </is>
@@ -1888,15 +2046,20 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
+          <t>And may Rudā take vengeance on his enemy.</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>By ʿMrt son of ʿBd son of Ḥrm, and may Rudā take vengeance on his enemy.</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
           <t>l-ʿmrt bn ʿbd bn ḥrm w-h-Rudā nqm mn s²nʾ-h</t>
         </is>
       </c>
-      <c r="F6" s="11" t="inlineStr">
-        <is>
-          <t>By ʿMrt son of ʿBd son of Ḥrm, and may Rudā take vengeance on his enemy.</t>
-        </is>
-      </c>
-      <c r="G6" s="11" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>RSIS0002.xml</t>
         </is>
@@ -1913,7 +2076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1922,7 +2085,8 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1948,15 +2112,20 @@
       </c>
       <c r="E1" s="6" t="inlineStr">
         <is>
+          <t>Invocation (English)</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Full Translation</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
           <t>Safaitic Text (Transliteration)</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
-        <is>
-          <t>English Translation</t>
-        </is>
-      </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Source File</t>
         </is>
@@ -1985,15 +2154,20 @@
       </c>
       <c r="E2" s="12" t="inlineStr">
         <is>
+          <t>And may Shams grant him good fortune and (good) pasture and rain.</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>By ʿWr son of Ngr, and may Shams grant him good fortune and (good) pasture and rain.</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
           <t>l-ʿwr bn ngr w-h-Šms tns¹ʿd-h w-mrʿ w-wbl</t>
         </is>
       </c>
-      <c r="F2" s="12" t="inlineStr">
-        <is>
-          <t>By ʿWr son of Ngr, and may Shams grant him good fortune and (good) pasture and rain.</t>
-        </is>
-      </c>
-      <c r="G2" s="12" t="inlineStr">
+      <c r="H2" s="12" t="inlineStr">
         <is>
           <t>USMF0001.xml</t>
         </is>
@@ -2022,15 +2196,20 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
+          <t>And may Shams (grant) rain and good pasture for his camels.</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>By Sʿd son of Ġwt, while he pastured the camels, and may Shams (grant) rain and good pasture for his camels.</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
           <t>l-s¹ʿd bn ġwt w-rʿy h-ibl w-h-Šms gyt w-mrʿ l-ibl-h</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>By Sʿd son of Ġwt, while he pastured the camels, and may Shams (grant) rain and good pasture for his camels.</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>HCH0002.xml</t>
         </is>
@@ -2059,15 +2238,20 @@
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
+          <t>And may Shams (grant) good pasture and rain.</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>By Ṯʿlbt son of Slm, while he pastured the sheep, and may Shams (grant) good pasture and rain.</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
           <t>l-ṯʿlbt bn s¹lm w-rʿy h-ġnm w-h-Šms mrʿ w-gyt</t>
         </is>
       </c>
-      <c r="F4" s="12" t="inlineStr">
-        <is>
-          <t>By Ṯʿlbt son of Slm, while he pastured the sheep, and may Shams (grant) good pasture and rain.</t>
-        </is>
-      </c>
-      <c r="G4" s="12" t="inlineStr">
+      <c r="H4" s="12" t="inlineStr">
         <is>
           <t>HCH0003.xml</t>
         </is>
@@ -2096,15 +2280,20 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
+          <t>And may Shams (grant) good pasture and rain and gain.</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>By Ġnm son of ʿMr, while he pastured (flocks), and may Shams (grant) good pasture and rain and gain.</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
           <t>l-ġnm bn ʿmr w-rʿy w-h-Šms mrʿ w-gyt w-ks²b</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>By Ġnm son of ʿMr, while he pastured (flocks), and may Shams (grant) good pasture and rain and gain.</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>WH0002.xml</t>
         </is>
@@ -2121,7 +2310,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2130,7 +2319,8 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -2156,15 +2346,20 @@
       </c>
       <c r="E1" s="7" t="inlineStr">
         <is>
+          <t>Invocation (English)</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>Full Translation</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
           <t>Safaitic Text (Transliteration)</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
-        <is>
-          <t>English Translation</t>
-        </is>
-      </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Source File</t>
         </is>
@@ -2193,15 +2388,20 @@
       </c>
       <c r="E2" s="13" t="inlineStr">
         <is>
+          <t>And may Allāt (grant) protection, and may Rudā take vengeance on his enemy, and may Shams (grant) rain and good pasture.</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="inlineStr">
+        <is>
+          <t>By Ṣhr son of Sʿd son of Ṯlm, and may Allāt (grant) protection, and may Rudā take vengeance on his enemy, and may Shams (grant) rain and good pasture.</t>
+        </is>
+      </c>
+      <c r="G2" s="13" t="inlineStr">
+        <is>
           <t>l-ṣhr bn s¹ʿd bn ṯlm w-h-Allāt ḥmyt w-h-Rudā nqm mn s²nʾ-h w-h-Šms gyt w-mrʿ</t>
         </is>
       </c>
-      <c r="F2" s="13" t="inlineStr">
-        <is>
-          <t>By Ṣhr son of Sʿd son of Ṯlm, and may Allāt (grant) protection, and may Rudā take vengeance on his enemy, and may Shams (grant) rain and good pasture.</t>
-        </is>
-      </c>
-      <c r="G2" s="13" t="inlineStr">
+      <c r="H2" s="13" t="inlineStr">
         <is>
           <t>USMF0003.xml</t>
         </is>
@@ -2230,15 +2430,20 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
+          <t>And may Allāt (grant) protection, and may Rudā take vengeance for him on his enemy, and may Shams (grant) good pasture.</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>By Ḥry son of ʿMr son of ʿBd, and may Allāt (grant) protection, and may Rudā take vengeance for him on his enemy, and may Shams (grant) good pasture.</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
           <t>l-ḥry bn ʿmr bn ʿbd w-h-Allāt ḥmyt w-h-Rudā nqm l-h mn ʿdw-h w-h-Šms mrʿ</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>By Ḥry son of ʿMr son of ʿBd, and may Allāt (grant) protection, and may Rudā take vengeance for him on his enemy, and may Shams (grant) good pasture.</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>KRS0003.xml</t>
         </is>
@@ -2267,15 +2472,20 @@
       </c>
       <c r="E4" s="13" t="inlineStr">
         <is>
+          <t>And may Shams (grant) good pasture and rain and gain, and may Allāt (grant) protection.</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>By ʿBd-Šms son of Mlk, while he pastured (flocks), and may Shams (grant) good pasture and rain and gain, and may Allāt (grant) protection.</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
           <t>l-ʿbd- Šms bn mlk w-rʿy w-h-Šms mrʿ w-wbl w-ks²b w-h-Allāt ḥmyt</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
-        <is>
-          <t>By ʿBd-Šms son of Mlk, while he pastured (flocks), and may Shams (grant) good pasture and rain and gain, and may Allāt (grant) protection.</t>
-        </is>
-      </c>
-      <c r="G4" s="13" t="inlineStr">
+      <c r="H4" s="13" t="inlineStr">
         <is>
           <t>JDWS0002.xml</t>
         </is>
@@ -2304,15 +2514,20 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
+          <t>And may Allāt protect him from every enemy, and may Shams (grant) pasture and gain.</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>By Ḥnn son of Ṣhr, and may Allāt protect him from every enemy, and may Shams (grant) pasture and gain.</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
           <t>l-ḥnn bn ṣhr w-h-Allāt ḥmy-h mn kl ʿdw w-h-Šms mrʿ w-ks²b</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>By Ḥnn son of Ṣhr, and may Allāt protect him from every enemy, and may Shams (grant) pasture and gain.</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>RSIS0001.xml</t>
         </is>
@@ -2341,15 +2556,20 @@
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
+          <t>And may Allāt take vengeance for him on his enemy, and may Rudā protect him.</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>By Ṯlm son of Ḫlf son of Šbq, and may Allāt take vengeance for him on his enemy, and may Rudā protect him.</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
           <t>l-ṯlm bn ḫlf bn s²bq w-h-Allāt nqm-h mn s²nʾ-h w-h-Rudā ḥmy-h</t>
         </is>
       </c>
-      <c r="F6" s="13" t="inlineStr">
-        <is>
-          <t>By Ṯlm son of Ḫlf son of Šbq, and may Allāt take vengeance for him on his enemy, and may Rudā protect him.</t>
-        </is>
-      </c>
-      <c r="G6" s="13" t="inlineStr">
+      <c r="H6" s="13" t="inlineStr">
         <is>
           <t>WH0003.xml</t>
         </is>

</xml_diff>